<commit_message>
docs: update status tracker
</commit_message>
<xml_diff>
--- a/docs/StatusTracker.xlsx
+++ b/docs/StatusTracker.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="141">
   <si>
     <t xml:space="preserve">Using the Status tracker</t>
   </si>
@@ -453,10 +453,16 @@
     <t xml:space="preserve">Offline Client Meeting</t>
   </si>
   <si>
+    <t xml:space="preserve">Implement new TermExtractor</t>
+  </si>
+  <si>
     <t xml:space="preserve">Code refactoring</t>
   </si>
   <si>
-    <t xml:space="preserve">Advait, Amish, Keshav</t>
+    <t xml:space="preserve">Refactor Backend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interactive CLI Demos</t>
   </si>
   <si>
     <t xml:space="preserve">Client Office Visit</t>
@@ -472,6 +478,9 @@
   </si>
   <si>
     <t xml:space="preserve">Updated requirements document</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Made R2 Presentation</t>
   </si>
 </sst>
 </file>
@@ -483,7 +492,7 @@
     <numFmt numFmtId="165" formatCode="General"/>
     <numFmt numFmtId="166" formatCode="@"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -569,12 +578,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -639,7 +642,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -765,10 +768,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2170,7 +2169,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z1022"/>
+  <dimension ref="A1:Z1025"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="2" outlineLevelCol="1"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="1" min="1" style="1" width="60.5"/>
@@ -3780,7 +3779,7 @@
       <c r="B66" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C66" s="32" t="s">
+      <c r="C66" s="2" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="2" t="n">
@@ -3808,7 +3807,7 @@
       <c r="B67" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C67" s="32" t="s">
+      <c r="C67" s="2" t="s">
         <v>119</v>
       </c>
       <c r="D67" s="2" t="n">
@@ -3848,7 +3847,7 @@
       <c r="B69" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C69" s="32" t="s">
+      <c r="C69" s="2" t="s">
         <v>54</v>
       </c>
       <c r="D69" s="2" t="n">
@@ -3967,7 +3966,7 @@
       <c r="F74" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="G74" s="33" t="s">
+      <c r="G74" s="32" t="s">
         <v>125</v>
       </c>
       <c r="H74" s="26"/>
@@ -4057,7 +4056,7 @@
       <c r="B79" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C79" s="32" t="s">
+      <c r="C79" s="2" t="s">
         <v>36</v>
       </c>
       <c r="D79" s="2" t="n">
@@ -4080,63 +4079,61 @@
     </row>
     <row r="80" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
-        <v>48</v>
+        <v>131</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>37</v>
+        <v>54</v>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>0.3</v>
+        <v>6</v>
       </c>
       <c r="F80" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H80" s="26" t="e">
-        <f aca="false">IF(OR(D80="",E80=""),"",D80-E80)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I80" s="26" t="e">
-        <f aca="false">IF(OR(H80="",E80=0),"",ABS(H80)/E80*100)</f>
-        <v>#VALUE!</v>
-      </c>
+      <c r="H80" s="26"/>
+      <c r="I80" s="26"/>
     </row>
     <row r="81" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B81" s="4"/>
+        <v>48</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>45</v>
+      </c>
       <c r="C81" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D81" s="2" t="n">
-        <v>1</v>
+        <v>49</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>1.5</v>
+        <v>0.3</v>
       </c>
       <c r="F81" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H81" s="26" t="n">
+      <c r="H81" s="26" t="e">
         <f aca="false">IF(OR(D81="",E81=""),"",D81-E81)</f>
-        <v>-0.5</v>
-      </c>
-      <c r="I81" s="26" t="n">
+        <v>#VALUE!</v>
+      </c>
+      <c r="I81" s="26" t="e">
         <f aca="false">IF(OR(H81="",E81=0),"",ABS(H81)/E81*100)</f>
-        <v>33.3333333333333</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B82" s="4"/>
+      <c r="B82" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="C82" s="2" t="s">
         <v>89</v>
       </c>
@@ -4160,13 +4157,13 @@
     </row>
     <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>78</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>132</v>
+        <v>63</v>
       </c>
       <c r="D83" s="2" t="n">
         <v>2</v>
@@ -4191,10 +4188,10 @@
         <v>133</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="D84" s="2" t="n">
         <v>3</v>
@@ -4205,58 +4202,46 @@
       <c r="F84" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H84" s="26" t="n">
-        <f aca="false">IF(OR(D84="",E84=""),"",D84-E84)</f>
-        <v>0</v>
-      </c>
-      <c r="I84" s="26" t="n">
-        <f aca="false">IF(OR(H84="",E84=0),"",ABS(H84)/E84*100)</f>
-        <v>0</v>
-      </c>
+      <c r="H84" s="26"/>
+      <c r="I84" s="26"/>
     </row>
     <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="D85" s="2" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F85" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H85" s="26" t="n">
-        <f aca="false">IF(OR(D85="",E85=""),"",D85-E85)</f>
-        <v>0</v>
-      </c>
-      <c r="I85" s="26" t="n">
-        <f aca="false">IF(OR(H85="",E85=0),"",ABS(H85)/E85*100)</f>
-        <v>0</v>
-      </c>
+      <c r="H85" s="26"/>
+      <c r="I85" s="26"/>
     </row>
     <row r="86" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
         <v>135</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>96</v>
+        <v>35</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>119</v>
+        <v>36</v>
       </c>
       <c r="D86" s="2" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="F86" s="8" t="s">
         <v>38</v>
@@ -4278,7 +4263,7 @@
         <v>45</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="D87" s="2" t="n">
         <v>0.5</v>
@@ -4303,16 +4288,16 @@
         <v>137</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>45</v>
+        <v>96</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>60</v>
+        <v>119</v>
       </c>
       <c r="D88" s="2" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F88" s="8" t="s">
         <v>38</v>
@@ -4327,11 +4312,11 @@
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="4" t="s">
-        <v>92</v>
+      <c r="A89" s="1" t="s">
+        <v>138</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>60</v>
@@ -4355,49 +4340,82 @@
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B90" s="4"/>
-      <c r="C90" s="2"/>
-      <c r="D90" s="2"/>
-      <c r="E90" s="2"/>
-      <c r="F90" s="8"/>
-      <c r="H90" s="26" t="str">
+      <c r="A90" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F90" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="H90" s="26" t="n">
         <f aca="false">IF(OR(D90="",E90=""),"",D90-E90)</f>
-        <v/>
-      </c>
-      <c r="I90" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="I90" s="26" t="n">
         <f aca="false">IF(OR(H90="",E90=0),"",ABS(H90)/E90*100)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B91" s="4"/>
-      <c r="C91" s="2"/>
-      <c r="D91" s="2"/>
-      <c r="E91" s="2"/>
-      <c r="F91" s="8"/>
-      <c r="H91" s="26" t="str">
+      <c r="A91" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F91" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="H91" s="26" t="n">
         <f aca="false">IF(OR(D91="",E91=""),"",D91-E91)</f>
-        <v/>
-      </c>
-      <c r="I91" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="I91" s="26" t="n">
         <f aca="false">IF(OR(H91="",E91=0),"",ABS(H91)/E91*100)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B92" s="4"/>
-      <c r="C92" s="2"/>
-      <c r="D92" s="2"/>
-      <c r="E92" s="2"/>
-      <c r="F92" s="8"/>
-      <c r="H92" s="26" t="str">
-        <f aca="false">IF(OR(D92="",E92=""),"",D92-E92)</f>
-        <v/>
-      </c>
-      <c r="I92" s="26" t="str">
-        <f aca="false">IF(OR(H92="",E92=0),"",ABS(H92)/E92*100)</f>
-        <v/>
-      </c>
+      <c r="A92" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E92" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F92" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="H92" s="26"/>
+      <c r="I92" s="26"/>
     </row>
     <row r="93" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B93" s="4"/>
@@ -6760,7 +6778,10 @@
       <c r="D250" s="2"/>
       <c r="E250" s="2"/>
       <c r="F250" s="8"/>
-      <c r="H250" s="9"/>
+      <c r="H250" s="26" t="str">
+        <f aca="false">IF(OR(D250="",E250=""),"",D250-E250)</f>
+        <v/>
+      </c>
       <c r="I250" s="26" t="str">
         <f aca="false">IF(OR(H250="",E250=0),"",ABS(H250)/E250*100)</f>
         <v/>
@@ -6772,7 +6793,10 @@
       <c r="D251" s="2"/>
       <c r="E251" s="2"/>
       <c r="F251" s="8"/>
-      <c r="H251" s="9"/>
+      <c r="H251" s="26" t="str">
+        <f aca="false">IF(OR(D251="",E251=""),"",D251-E251)</f>
+        <v/>
+      </c>
       <c r="I251" s="26" t="str">
         <f aca="false">IF(OR(H251="",E251=0),"",ABS(H251)/E251*100)</f>
         <v/>
@@ -6784,7 +6808,10 @@
       <c r="D252" s="2"/>
       <c r="E252" s="2"/>
       <c r="F252" s="8"/>
-      <c r="H252" s="9"/>
+      <c r="H252" s="26" t="str">
+        <f aca="false">IF(OR(D252="",E252=""),"",D252-E252)</f>
+        <v/>
+      </c>
       <c r="I252" s="26" t="str">
         <f aca="false">IF(OR(H252="",E252=0),"",ABS(H252)/E252*100)</f>
         <v/>
@@ -6845,7 +6872,10 @@
       <c r="E257" s="2"/>
       <c r="F257" s="8"/>
       <c r="H257" s="9"/>
-      <c r="I257" s="9"/>
+      <c r="I257" s="26" t="str">
+        <f aca="false">IF(OR(H257="",E257=0),"",ABS(H257)/E257*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="258" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B258" s="4"/>
@@ -6854,7 +6884,10 @@
       <c r="E258" s="2"/>
       <c r="F258" s="8"/>
       <c r="H258" s="9"/>
-      <c r="I258" s="9"/>
+      <c r="I258" s="26" t="str">
+        <f aca="false">IF(OR(H258="",E258=0),"",ABS(H258)/E258*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="259" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B259" s="4"/>
@@ -6863,7 +6896,10 @@
       <c r="E259" s="2"/>
       <c r="F259" s="8"/>
       <c r="H259" s="9"/>
-      <c r="I259" s="9"/>
+      <c r="I259" s="26" t="str">
+        <f aca="false">IF(OR(H259="",E259=0),"",ABS(H259)/E259*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="260" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B260" s="4"/>
@@ -8638,17 +8674,32 @@
       <c r="H456" s="9"/>
       <c r="I456" s="9"/>
     </row>
-    <row r="457" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="457" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B457" s="4"/>
-      <c r="F457" s="4"/>
-    </row>
-    <row r="458" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C457" s="2"/>
+      <c r="D457" s="2"/>
+      <c r="E457" s="2"/>
+      <c r="F457" s="8"/>
+      <c r="H457" s="9"/>
+      <c r="I457" s="9"/>
+    </row>
+    <row r="458" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B458" s="4"/>
-      <c r="F458" s="4"/>
-    </row>
-    <row r="459" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C458" s="2"/>
+      <c r="D458" s="2"/>
+      <c r="E458" s="2"/>
+      <c r="F458" s="8"/>
+      <c r="H458" s="9"/>
+      <c r="I458" s="9"/>
+    </row>
+    <row r="459" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B459" s="4"/>
-      <c r="F459" s="4"/>
+      <c r="C459" s="2"/>
+      <c r="D459" s="2"/>
+      <c r="E459" s="2"/>
+      <c r="F459" s="8"/>
+      <c r="H459" s="9"/>
+      <c r="I459" s="9"/>
     </row>
     <row r="460" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B460" s="4"/>
@@ -10902,8 +10953,20 @@
       <c r="B1022" s="4"/>
       <c r="F1022" s="4"/>
     </row>
+    <row r="1023" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1023" s="4"/>
+      <c r="F1023" s="4"/>
+    </row>
+    <row r="1024" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1024" s="4"/>
+      <c r="F1024" s="4"/>
+    </row>
+    <row r="1025" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1025" s="4"/>
+      <c r="F1025" s="4"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="F5:F21 F23:F38 F40:F44 F47:F58 F60 F62 F64 F66:F69 F79:F1022 F71:F77">
+  <conditionalFormatting sqref="F5:F21 F23:F38 F40:F44 F47:F58 F60 F62 F64 F66:F69 F79:F1025 F71:F77">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Delayed"</formula>
     </cfRule>
@@ -10960,11 +11023,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" prompt=" - " showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F5:F45 F47:F58 F60 F62 F64 F66:F69 F71:F77 F79:F1022" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" prompt=" - " showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F5:F45 F47:F58 F60 F62 F64 F66:F69 F71:F77 F79:F1025" type="list">
       <formula1>"Planned,Ongoing,Delayed,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" prompt=" - " showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B5:B45 B47:B58 B60 B62 B64 B66:B69 B71:B77 B79:B1022" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" prompt=" - " showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B5:B45 B47:B58 B60 B62 B64 B66:B69 B71:B77 B79:B1025" type="list">
       <formula1>"Requirements,Design,Development,Testing,Preparation,Coordination,Documentation,Interfaces,Delivery"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>